<commit_message>
Daily auto backup 2026-08-12 17:10
</commit_message>
<xml_diff>
--- a/check.xlsx
+++ b/check.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,51 +506,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7040622</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>BM-00105824</t>
-        </is>
-      </c>
+          <t>6649716</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rukhsana Tabassum (MS/EBV5-SWC)</t>
+          <t>Ben Khelifa Hichem (VM/ESB4)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>50000</v>
+        <v>93.48</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>22-05-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>17-06-2026</t>
+          <t>07-04-2026</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -565,19 +561,23 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>6988136</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+          <t>7040622</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BM-00105824</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mohamed Arsath B (MS/PJ-CISW1-VM)</t>
+          <t>Rukhsana Tabassum (MS/EBV5-SWC)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -586,16 +586,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>50000</v>
+        <v>26.71</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>08-05-2026</t>
+          <t>22-05-2026</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>22-05-2026</t>
+          <t>17-06-2026</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -605,13 +605,13 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.25</v>
+        <v>13</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.25</v>
+        <v>13</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -626,37 +626,37 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7040751</t>
+          <t>7083721</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Heid Dimitrij (VM/ESB4)</t>
+          <t>Abishek Boraian (MS/EMB1-VM)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>India</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>175000</v>
+        <v>26.71</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>22-05-2026</t>
+          <t>03-06-2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>No Date</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -666,13 +666,13 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
@@ -687,7 +687,7 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>50000</v>
+        <v>26.71</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -754,62 +754,550 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6649716</t>
+          <t>6988136</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ben Khelifa Hichem (VM/ESB4)</t>
+          <t>Mohamed Arsath B (MS/PJ-CISW1-VM)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>08-05-2026</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>22-05-2026</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7040751</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Heid Dimitrij (VM/ESB4)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>175000</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>05-02-2026</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>07-04-2026</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>4</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
+      <c r="E7" t="n">
+        <v>93.48</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>22-05-2026</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>6960725</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Akash Bhaskara Mogaveera (MS/EHE2-VM)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>29-04-2026</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>No Date</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>18</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>18</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5833959</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Majhi Shouvik (MS/EBV3-SWC)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>18-06-2025</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>18-07-2025</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>126.5</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>126.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6806296</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Adithya Krishnan (MS/EBV3-SWC)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>23-03-2026</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>01-07-2026</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>494.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>735.5700000000001</v>
+      </c>
+      <c r="J10" t="n">
+        <v>261.5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>508.7</v>
+      </c>
+      <c r="L10" t="n">
+        <v>997.0700000000001</v>
+      </c>
+      <c r="M10" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>997.0700000000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6806296</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>To Giang Tuan Anh (MS/EHV12-VM)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>22.73</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>23-03-2026</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>01-07-2026</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>96</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>96</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>6806296</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Heid Dimitrij (VM/ESB4)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>93.48</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>23-03-2026</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>01-07-2026</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>16.88</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>16.88</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>16.88</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>6806300</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Rukhsana Tabassum (MS/EBV5-SWC)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>23-03-2026</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>10-07-2026</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>550.85</v>
+      </c>
+      <c r="I13" t="n">
+        <v>315.65</v>
+      </c>
+      <c r="J13" t="n">
+        <v>280.5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>555.85</v>
+      </c>
+      <c r="L13" t="n">
+        <v>596.15</v>
+      </c>
+      <c r="M13" t="n">
+        <v>5</v>
+      </c>
+      <c r="N13" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="O13" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="P13" t="n">
+        <v>57.25</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>653.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>6806300</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Heid Dimitrij (VM/ESB4)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>93.48</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>23-03-2026</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>10-07-2026</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="K14" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="L14" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="P14" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily auto backup 2026-08-14 09:49
</commit_message>
<xml_diff>
--- a/check.xlsx
+++ b/check.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,35 +506,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6649716</t>
+          <t>7083721</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ben Khelifa Hichem (VM/ESB4)</t>
+          <t>Abishek Boraian (MS/EMB1-VM)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>India</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>93.48</v>
+        <v>26.71</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>03-06-2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>07-04-2026</t>
+          <t>No Date</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -543,7 +543,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -567,17 +567,13 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7040622</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>BM-00105824</t>
-        </is>
-      </c>
+          <t>6988136</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Rukhsana Tabassum (MS/EBV5-SWC)</t>
+          <t>Mohamed Arsath B (MS/PJ-CISW1-VM)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -590,14 +586,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>08-05-2026</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>22-05-2026</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>17-06-2026</t>
-        </is>
-      </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
@@ -605,13 +601,13 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>13</v>
+        <v>0.25</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>13</v>
+        <v>0.25</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -626,41 +622,41 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>13</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7083721</t>
+          <t>6649716</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Abishek Boraian (MS/EMB1-VM)</t>
+          <t>Ben Khelifa Hichem (VM/ESB4)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>26.71</v>
+        <v>93.48</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>03-06-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No Date</t>
+          <t>07-04-2026</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -669,7 +665,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -693,13 +689,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7040712</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>7040622</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BM-00105824</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mohamed Arsath B (MS/PJ-CISW1-VM)</t>
+          <t>Rukhsana Tabassum (MS/EBV5-SWC)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>17-06-2026</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -727,13 +727,13 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>48.5</v>
+        <v>13</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>48.5</v>
+        <v>13</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -748,13 +748,13 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>48.5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6988136</t>
+          <t>7040712</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -773,12 +773,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08-05-2026</t>
+          <t>22-05-2026</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>22-05-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -788,13 +788,13 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.25</v>
+        <v>48.5</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0.25</v>
+        <v>48.5</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
@@ -809,7 +809,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.25</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="7">
@@ -998,7 +998,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6806296</t>
+          <t>5680751</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -1017,31 +1017,31 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>23-03-2026</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>494.2</v>
+        <v>51.5</v>
       </c>
       <c r="I10" t="n">
-        <v>735.5700000000001</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>261.5</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>508.7</v>
+        <v>51.5</v>
       </c>
       <c r="L10" t="n">
-        <v>997.0700000000001</v>
+        <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -1053,56 +1053,56 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>997.0700000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6806296</t>
+          <t>5680751</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>To Giang Tuan Anh (MS/EHV12-VM)</t>
+          <t>Brueggemann Joerg (VM/ESB4)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>22.73</v>
+        <v>93.48</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>23-03-2026</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I11" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="L11" t="n">
-        <v>96</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -1114,53 +1114,53 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6806296</t>
+          <t>5680742</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Heid Dimitrij (VM/ESB4)</t>
+          <t>Anant R K Ashwin (MS/EHE2-VM)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>India</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>93.48</v>
+        <v>26.71</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>23-03-2026</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>197.5</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>348.24</v>
       </c>
       <c r="J12" t="n">
-        <v>16.88</v>
+        <v>23.5</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>197.5</v>
       </c>
       <c r="L12" t="n">
-        <v>16.88</v>
+        <v>371.74</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -1175,129 +1175,922 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>16.88</v>
+        <v>371.74</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>6806300</t>
+          <t>5680742</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Rukhsana Tabassum (MS/EBV5-SWC)</t>
+          <t>Elamari Taoufik (VM/ESB4)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>26.71</v>
+        <v>93.48</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>23-03-2026</t>
+          <t>29-04-2025</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>550.85</v>
+        <v>137.5</v>
       </c>
       <c r="I13" t="n">
-        <v>315.65</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>280.5</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>555.85</v>
+        <v>137.5</v>
       </c>
       <c r="L13" t="n">
-        <v>596.15</v>
+        <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>18.75</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>38.5</v>
+        <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>57.25</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>653.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>6806300</t>
+          <t>5680742</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
+          <t>Lima Rui (VM/ESE1-Brg)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>42.74</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>29-04-2025</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>22-10-2025</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>12</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>12</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>6806296</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Adithya Krishnan (MS/EBV3-SWC)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>23-03-2026</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>01-07-2026</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>494.2</v>
+      </c>
+      <c r="I15" t="n">
+        <v>735.5700000000001</v>
+      </c>
+      <c r="J15" t="n">
+        <v>261.5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>508.7</v>
+      </c>
+      <c r="L15" t="n">
+        <v>997.0700000000001</v>
+      </c>
+      <c r="M15" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>997.0700000000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>6806296</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>To Giang Tuan Anh (MS/EHV12-VM)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>22.73</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>23-03-2026</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>01-07-2026</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>96</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>96</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>6806296</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>Heid Dimitrij (VM/ESB4)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E17" t="n">
         <v>93.48</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>23-03-2026</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>01-07-2026</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>16.88</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>16.88</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>16.88</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>6806300</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Rukhsana Tabassum (MS/EBV5-SWC)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>23-03-2026</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
         <is>
           <t>10-07-2026</t>
         </is>
       </c>
-      <c r="H14" t="n">
+      <c r="H18" t="n">
+        <v>550.85</v>
+      </c>
+      <c r="I18" t="n">
+        <v>315.65</v>
+      </c>
+      <c r="J18" t="n">
+        <v>280.5</v>
+      </c>
+      <c r="K18" t="n">
+        <v>555.85</v>
+      </c>
+      <c r="L18" t="n">
+        <v>596.15</v>
+      </c>
+      <c r="M18" t="n">
+        <v>5</v>
+      </c>
+      <c r="N18" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="O18" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="P18" t="n">
+        <v>57.25</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>653.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>6806300</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Heid Dimitrij (VM/ESB4)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>93.48</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>23-03-2026</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>10-07-2026</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
         <v>15.9</v>
       </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
         <v>5.25</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K19" t="n">
         <v>15.9</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L19" t="n">
         <v>5.25</v>
       </c>
-      <c r="M14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="n">
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
         <v>2.75</v>
       </c>
-      <c r="P14" t="n">
+      <c r="P19" t="n">
         <v>2.75</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q19" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>5417327</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Abishek K S D (MS/EHE2-VM)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>13-02-2025</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>31-03-2026</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>232</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1118.4</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>316.5</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1118.4</v>
+      </c>
+      <c r="M20" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="N20" t="n">
+        <v>214.75</v>
+      </c>
+      <c r="O20" t="n">
+        <v>4</v>
+      </c>
+      <c r="P20" t="n">
+        <v>218.75</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>1337.15</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>5417327</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>EXTERNAL Ramamurthy Ragavi (T&amp;amp;S (Technology and Strategy), VM/ESB3-CB)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>93.48</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>13-02-2025</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>31-03-2026</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>215</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>215</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>45</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>5417327</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Filsinger Felix (VM/EAE3-CB)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>13-02-2025</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>31-03-2026</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>5500147</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lakkoju Veera Venkata Naga Sri Charan (MS/EBV3-SWC)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>07-03-2025</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>27-03-2026</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>365.75</v>
+      </c>
+      <c r="I23" t="n">
+        <v>293</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>482</v>
+      </c>
+      <c r="L23" t="n">
+        <v>293</v>
+      </c>
+      <c r="M23" t="n">
+        <v>116.25</v>
+      </c>
+      <c r="N23" t="n">
+        <v>59.75</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>59.75</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>352.75</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>5500147</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>EXTERNAL Balakrishnan Vengatesh (Technology and Strategy (TS), VM/ECE2-CB)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>93.48</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>07-03-2025</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>27-03-2026</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>194</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>194</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>63</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>63</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>5500147</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Nguyen Thanh Phuc (MS/EHV12-VM)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>22.73</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>07-03-2025</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>27-03-2026</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>38</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>38</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>5500149</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Anitha Anju (MS/EHE2-VM)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>07-03-2025</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>06-04-2026</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>892.1</v>
+      </c>
+      <c r="I26" t="n">
+        <v>816</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1155.85</v>
+      </c>
+      <c r="L26" t="n">
+        <v>816</v>
+      </c>
+      <c r="M26" t="n">
+        <v>263.75</v>
+      </c>
+      <c r="N26" t="n">
+        <v>292.25</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>292.25</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>1108.25</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>5500149</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>EXTERNAL Balakrishnan Vengatesh (Technology and Strategy (TS), VM/ECE2-CB)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>93.48</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>07-03-2025</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>06-04-2026</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>621.25</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>621.25</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>666.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>